<commit_message>
Daily slate 2026-06-07 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-05.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-05.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F2" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G2" t="n">
-        <v>42</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E3" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F3" t="n">
         <v>93</v>
       </c>
       <c r="G3" t="n">
-        <v>49.5</v>
+        <v>49.7</v>
       </c>
     </row>
     <row r="4">
@@ -529,13 +529,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4" t="n">
         <v>33.3</v>
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E5" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F5" t="n">
         <v>83</v>
       </c>
       <c r="G5" t="n">
-        <v>41.1</v>
+        <v>42.4</v>
       </c>
     </row>
     <row r="6">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
         <v>5</v>
       </c>
       <c r="G7" t="n">
-        <v>61.5</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="8">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1125</v>
+        <v>1170</v>
       </c>
       <c r="E11" t="n">
-        <v>681</v>
+        <v>704</v>
       </c>
       <c r="F11" t="n">
-        <v>444</v>
+        <v>466</v>
       </c>
       <c r="G11" t="n">
-        <v>60.5</v>
+        <v>60.2</v>
       </c>
     </row>
     <row r="12">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="E14" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F14" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="G14" t="n">
-        <v>25.7</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="E15" t="n">
         <v>72</v>
       </c>
       <c r="F15" t="n">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="G15" t="n">
-        <v>18.2</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="E16" t="n">
         <v>53</v>
       </c>
       <c r="F16" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G16" t="n">
-        <v>27.2</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4801</v>
+        <v>5002</v>
       </c>
       <c r="E17" t="n">
-        <v>1085</v>
+        <v>1117</v>
       </c>
       <c r="F17" t="n">
-        <v>3716</v>
+        <v>3885</v>
       </c>
       <c r="G17" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
     </row>
   </sheetData>
@@ -1558,10 +1558,10 @@
         <v>221</v>
       </c>
       <c r="D7" t="n">
-        <v>60.5</v>
+        <v>60.2</v>
       </c>
       <c r="E7" t="n">
-        <v>1125</v>
+        <v>1170</v>
       </c>
       <c r="F7" t="n">
         <v>63.4</v>
@@ -1576,40 +1576,40 @@
         <v>227</v>
       </c>
       <c r="J7" t="n">
-        <v>25.7</v>
+        <v>25.3</v>
       </c>
       <c r="K7" t="n">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="L7" t="n">
-        <v>18.2</v>
+        <v>17.8</v>
       </c>
       <c r="M7" t="n">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="N7" t="n">
-        <v>27.2</v>
+        <v>26.6</v>
       </c>
       <c r="O7" t="n">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="P7" t="n">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>4801</v>
+        <v>5002</v>
       </c>
       <c r="R7" t="n">
-        <v>42</v>
+        <v>41.9</v>
       </c>
       <c r="S7" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="T7" t="n">
         <v>33.3</v>
       </c>
       <c r="U7" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="V7" t="n">
         <v>56.6</v>
@@ -1624,22 +1624,22 @@
         <v>407</v>
       </c>
       <c r="Z7" t="n">
-        <v>49.5</v>
+        <v>49.7</v>
       </c>
       <c r="AA7" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AB7" t="n">
-        <v>41.1</v>
+        <v>42.4</v>
       </c>
       <c r="AC7" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="AD7" t="n">
-        <v>61.5</v>
+        <v>64.3</v>
       </c>
       <c r="AE7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AF7" t="n">
         <v>39.7</v>

</xml_diff>